<commit_message>
HU-017 native first: sai o Apex managed sharing e o LWC, entram Flow, sharing rules e Flow Test
</commit_message>
<xml_diff>
--- a/docs/hu017/HU017_Tarefas_Tecnicas.xlsx
+++ b/docs/hu017/HU017_Tarefas_Tecnicas.xlsx
@@ -24,7 +24,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">HU-017 - Tarefas Tecnicas - Busqueda y Gestion del Cliente Maestro en Salesforce</t>
+          <t xml:space="preserve">HU-017 - Tarefas Tecnicas - Busqueda y Gestion del Cliente Maestro en Salesforce. Native first: zero Apex e zero LWC</t>
         </is>
       </c>
     </row>
@@ -429,22 +429,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fluxo de extensao a outra sociedade</t>
+          <t xml:space="preserve">Tela de extensao a outra sociedade</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow ou LWC</t>
+          <t xml:space="preserve">Screen Flow</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extender cliente a sociedad</t>
+          <t xml:space="preserve">ExtendCustomerToSociety</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedir apenas os dados locais faltantes e criar o registro de relacao, sem gerar novo identificador maestro</t>
+          <t xml:space="preserve">Pedir apenas os dados locais faltantes e criar o registro de relacao, sem gerar novo identificador maestro. Usar componentes reativos, GA no Winter 24. Sem LWC. Se precisar de mais de uma sociedade por vez, avaliar o Repeater, lembrando que componente reativo nao funciona dentro dele</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1184,32 +1184,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visibilidade da conta por sociedade</t>
+          <t xml:space="preserve">OWD de Account privada</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">ApexClass</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountShare, compartilhamento gerido por Apex</t>
+          <t xml:space="preserve">Organization Wide Defaults</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWD de Account privada e compartilhamento calculado a partir dos registros de AccountAccountRelation. Restriction Rules nao cobrem Account e Sharing Rule so le campo da propria conta, que a RN-05 proibe</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T08</t>
+          <t xml:space="preserve">Deixar Account como Private. Sharing rule concede acesso e nunca restringe, entao sem OWD privada a RN-25 nao se sustenta</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25, CA-15, Escenario 7</t>
+          <t xml:space="preserve">RN-25, CA-15</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1221,37 +1216,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">T28</t>
+          <t xml:space="preserve">T27a</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo de permissoes e FLS</t>
+          <t xml:space="preserve">Verificar o operador do criterio de sharing rule</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">PermissionSet mais FLS</t>
+          <t xml:space="preserve">Verificacao</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">MasterDataAdmin, MasterDataRead</t>
+          <t xml:space="preserve">Setup, Sharing Settings</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separar quem administra o maestro de quem so cria e atualiza dentro do perfil, com FLS nos campos sensiveis</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T27</t>
+          <t xml:space="preserve">Abrir uma criteria-based sharing rule de Account e ver se o operador contains esta disponivel para campo texto. Decide entre um campo texto com 14 regras ou 14 checkbox com 14 regras</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-22, RN-25, CA-15</t>
+          <t xml:space="preserve">RN-25</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1263,12 +1253,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">T29</t>
+          <t xml:space="preserve">T27b</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca de nao sincronizado com SAP</t>
+          <t xml:space="preserve">Marca das sociedades habilitadas na conta</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1278,17 +1268,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account: estado de sincronizacao e ultimo erro</t>
+          <t xml:space="preserve">Account, um checkbox por sociedade, ou um texto com a lista</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcar o cliente como nao sincronizado quando a replicacao falhar. Usar o Nebula Logger para o erro, sem criar campo de log</t>
+          <t xml:space="preserve">Criar a marca que a sharing rule vai ler. Nao e a chave maestra, e derivado da AccountAccountRelation, entao nao conflita com a unicidade da RN-05. Confirmar essa leitura com a Melisa antes de empacotar</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27a</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-26, RN-27, CA-18, Escenario 8</t>
+          <t xml:space="preserve">RN-05, RN-25</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1300,37 +1295,37 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">T30</t>
+          <t xml:space="preserve">T27c</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atributos fiscais derivados por regra</t>
+          <t xml:space="preserve">Flow que estampa a marca de sociedade</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow ou ExpressionSet</t>
+          <t xml:space="preserve">Flow</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, derivacao automatica</t>
+          <t xml:space="preserve">AccountAccountRelation, apos criar, atualizar e excluir</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivar tipo de imposto, condicao de pagamento, classificacao B2C ou B2B, grupo de contas e lista de precos a partir do tipo de documento e de cliente. Nao se mostram na captura e sao sensiveis para a replicacao</t>
+          <t xml:space="preserve">Manter a marca da T27b sincronizada com os registros de relacao. E o contorno que a propria documentacao de sharing rule indica: automacao mantem o campo, a regra le o campo</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">T27b</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-32</t>
+          <t xml:space="preserve">RN-05, RN-25</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1342,44 +1337,74 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 4</t>
+          <t xml:space="preserve">T27d</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROTECAO DO DADO</t>
+          <t xml:space="preserve">Public group por sociedade</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Group</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Um public group por sociedade</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criar o grupo que recebe o acesso em cada regra, e definir quem entra em cada um</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-25</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">T31</t>
+          <t xml:space="preserve">T27e</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento de respaldo com principal</t>
+          <t xml:space="preserve">Criteria-based sharing rules por sociedade</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField mais Files</t>
+          <t xml:space="preserve">SharingRules</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, marcacao de documento principal</t>
+          <t xml:space="preserve">Account, uma regra por sociedade</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guardar identificacao, registro tributario e poderes como Files, com um campo que marque o principal. O expediente comercial e da HU-078</t>
+          <t xml:space="preserve">Uma regra por sociedade lendo a marca da T27b e concedendo ao grupo da T27d. Teto de 50 regras por criterio por objeto, e 14 sociedades cabem</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27b, T27c, T27d</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-31, CA-16</t>
+          <t xml:space="preserve">RN-25, Escenario 7</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1391,37 +1416,37 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">T27f</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ligar Data Protection and Privacy</t>
+          <t xml:space="preserve">Medir o recalculo de compartilhamento</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup</t>
+          <t xml:space="preserve">Verificacao</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objetos de consentimento</t>
+          <t xml:space="preserve">Antes da carga inicial</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Os objetos de consentimento so existem com a preferencia habilitada. Ligar antes de a HU-034 precisar</t>
+          <t xml:space="preserve">Atualizar a marca em volume dispara recalculo assincrono de compartilhamento. Medir com a base real antes da carga de clientes</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">T01</t>
+          <t xml:space="preserve">T27e</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-33</t>
+          <t xml:space="preserve">RN-25</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1433,37 +1458,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">T33</t>
+          <t xml:space="preserve">T28</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consentimento como dado do cliente</t>
+          <t xml:space="preserve">Modelo de permissoes e FLS</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reuso</t>
+          <t xml:space="preserve">PermissionSet mais FLS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Individual, ContactPointTypeConsent</t>
+          <t xml:space="preserve">MasterDataAdmin, MasterDataRead</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guardar consentimento e canal de preferencia nos objetos nativos. ContactPointTypeConsent tem BusinessBrandId, entao consentimento por marca sai nativo, o que importa num grupo multimarca</t>
+          <t xml:space="preserve">Separar quem administra o maestro de quem so cria e atualiza dentro do perfil, com FLS nos campos sensiveis</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">T27</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-33</t>
+          <t xml:space="preserve">RN-22, RN-25, CA-15</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1475,74 +1500,74 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">T34</t>
+          <t xml:space="preserve">T29</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarar o que depende de licenca nao contratada</t>
+          <t xml:space="preserve">Marca de nao sincronizado com SAP</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentacao</t>
+          <t xml:space="preserve">CustomField</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Riscos da HU</t>
+          <t xml:space="preserve">Account: estado de sincronizacao e ultimo erro</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cifrado at rest exige Shield e retencao com anonimizacao exige Privacy Center, nenhum dos dois licenciado. FLS e masking cobrem visibilidade e nao substituem cifra. Registrar como premissa, nao como tarefa</t>
+          <t xml:space="preserve">Marcar o cliente como nao sincronizado quando a replicacao falhar. Registrar o erro no Nebula Logger pela acao invocavel de Flow, sem escrever Apex e sem criar campo de log</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-29, RN-30</t>
+          <t xml:space="preserve">RN-26, RN-27, CA-18, Escenario 8</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOQUEADO</t>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T35</t>
+          <t xml:space="preserve">T30</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nao usar Dynamic Forms como seguranca</t>
+          <t xml:space="preserve">Atributos fiscais derivados por regra</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Padrao</t>
+          <t xml:space="preserve">Flow ou ExpressionSet</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisao das paginas</t>
+          <t xml:space="preserve">Account, derivacao automatica</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo escondido por regra de visibilidade continua acessivel em relatorio, list view e API. Proteger dado sensivel so por FLS</t>
+          <t xml:space="preserve">Derivar tipo de imposto, condicao de pagamento, classificacao B2C ou B2B, grupo de contas e lista de precos a partir do tipo de documento e de cliente. Nao se mostram na captura e sao sensiveis para a replicacao</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T19</t>
+          <t xml:space="preserve">T14</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-29</t>
+          <t xml:space="preserve">RN-32</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -1554,49 +1579,44 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 5</t>
+          <t xml:space="preserve">BLOCO 4</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">MULTI PAIS E FECHAMENTO</t>
+          <t xml:space="preserve">PROTECAO DO DADO</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">T36</t>
+          <t xml:space="preserve">T31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pais e dimensao de dado, nunca nome de metadado</t>
+          <t xml:space="preserve">Documento de respaldo com principal</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Padrao</t>
+          <t xml:space="preserve">CustomField mais Files</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisao de nomenclatura</t>
+          <t xml:space="preserve">Account, marcacao de documento principal</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">As regras por pais vivem nas tabelas do T14 e T15. Nenhum campo, flow ou classe com pais no API name</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">Guardar identificacao, registro tributario e poderes como Files, com um campo que marque o principal. O expediente comercial e da HU-078</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Convencao GRPQM</t>
+          <t xml:space="preserve">RN-31, CA-16</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -1608,37 +1628,37 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">T37</t>
+          <t xml:space="preserve">T32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
+          <t xml:space="preserve">Ligar Data Protection and Privacy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Translation</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Translation Workbench</t>
+          <t xml:space="preserve">Objetos de consentimento</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traduzir campos, valores de picklist, Record Types e mensagens de erro criados nesta HU</t>
+          <t xml:space="preserve">Os objetos de consentimento so existem com a preferencia habilitada. Ligar antes de a HU-034 precisar</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">T16</t>
+          <t xml:space="preserve">T01</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Convencao GRPQM</t>
+          <t xml:space="preserve">RN-33</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -1650,37 +1670,37 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">T38</t>
+          <t xml:space="preserve">T33</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order nos flows criados</t>
+          <t xml:space="preserve">Consentimento como dado do cliente</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Object Manager</t>
+          <t xml:space="preserve">Reuso</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order de cada flow em Account</t>
+          <t xml:space="preserve">Individual, ContactPointTypeConsent</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account ja e um dos objetos com mais automacao na org. Definir a ordem em cada flow novo</t>
+          <t xml:space="preserve">Guardar consentimento e canal de preferencia nos objetos nativos. ContactPointTypeConsent tem BusinessBrandId, entao consentimento por marca sai nativo, o que importa num grupo multimarca</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">T20</t>
+          <t xml:space="preserve">T32</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Governanca</t>
+          <t xml:space="preserve">RN-33</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -1692,40 +1712,257 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t xml:space="preserve">T34</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Declarar o que depende de licenca nao contratada</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentacao</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Riscos da HU</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cifrado at rest exige Shield e retencao com anonimizacao exige Privacy Center, nenhum dos dois licenciado. FLS e masking cobrem visibilidade e nao substituem cifra. Registrar como premissa, nao como tarefa</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-29, RN-30</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLOQUEADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T35</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nao usar Dynamic Forms como seguranca</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Padrao</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revisao das paginas</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Campo escondido por regra de visibilidade continua acessivel em relatorio, list view e API. Proteger dado sensivel so por FLS</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T19</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-29</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLOCO 5</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MULTI PAIS E FECHAMENTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T36</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pais e dimensao de dado, nunca nome de metadado</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Padrao</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revisao de nomenclatura</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As regras por pais vivem nas tabelas do T14 e T15. Nenhum campo, flow ou classe com pais no API name</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T14</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convencao GRPQM</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T37</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation Workbench</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir campos, valores de picklist, Record Types e mensagens de erro criados nesta HU</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T16</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convencao GRPQM</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T38</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trigger Order nos flows criados</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Object Manager</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trigger Order de cada flow em Account</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account ja e um dos objetos com mais automacao na org. Definir a ordem em cada flow novo</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T20</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Governanca</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t xml:space="preserve">T39</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t xml:space="preserve">Testes dos nove escenarios</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ApexClass</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Testes de unicidade, extensao e compartilhamento</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cobrir os escenarios 1 a 9, com enfase no 1, no 2 e no 7, que sao os que a RN-05 e a RN-25 tornam faceis de errar</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T27</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow Test</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Testes dos flows acionados por registro</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cobrir os escenarios 1 a 9 com Flow Test, que versiona junto com o flow. Enfase no 1, no 2 e no 7, e o 7 testado com usuario de outra sociedade, nunca com administrador</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27e</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t xml:space="preserve">A FAZER</t>
         </is>
@@ -1972,152 +2209,152 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">N08</t>
+          <t xml:space="preserve">N07b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-11, CA-06 obrigatorios por pais e tipo</t>
+          <t xml:space="preserve">RN-05, Escenario 2 tela de extensao</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic Forms</t>
+          <t xml:space="preserve">Screen Flow com componentes reativos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">REUSAR, SEM LWC</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suporta Person Account desde Winter 23 e permite comportamento Required condicional. Regra de secao so e avaliada depois de salvar, entao condicionar campo a campo</t>
+          <t xml:space="preserve">Reactive Screen Components GA no Winter 24 e Repeater no Spring 24, com pre carga no Winter 25. Componente reativo nao funciona dentro do Repeater</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">N09</t>
+          <t xml:space="preserve">N07c</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-12, RN-14, RN-21 regras por pais</t>
+          <t xml:space="preserve">Testes</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom Metadata Type</t>
+          <t xml:space="preserve">Flow Test</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONSTRUIR</t>
+          <t xml:space="preserve">REUSAR, SEM CLASSE DE TESTE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Editavel em Setup sem desenvolvimento, que e o que a RN-21 exige</t>
+          <t xml:space="preserve">Sem Apex nao ha classe de teste. Flow Test versiona junto com o flow</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">N10</t>
+          <t xml:space="preserve">N08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-13, CA-08 correio de faturacao</t>
+          <t xml:space="preserve">RN-11, CA-06 obrigatorios por pais e tipo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">ContactPointEmail</t>
+          <t xml:space="preserve">Dynamic Forms</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFICAR NO T01</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se existir, o tipo de uso separa faturacao de comercial sem criar campo</t>
+          <t xml:space="preserve">Suporta Person Account desde Winter 23 e permite comportamento Required condicional. Regra de secao so e avaliada depois de salvar, entao condicionar campo a campo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">N11</t>
+          <t xml:space="preserve">N09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-16, CA-11 chaves de coincidencia</t>
+          <t xml:space="preserve">RN-12, RN-14, RN-21 regras por pais</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Matching Rules</t>
+          <t xml:space="preserve">Custom Metadata Type</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">CONSTRUIR</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Esta HU define as chaves, a HU-006 configura</t>
+          <t xml:space="preserve">Editavel em Setup sem desenvolvimento, que e o que a RN-21 exige</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">N12</t>
+          <t xml:space="preserve">N10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-18 fusao de duplicados</t>
+          <t xml:space="preserve">RN-13, CA-08 correio de faturacao</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Merge nativo, inclusive Person Account</t>
+          <t xml:space="preserve">ContactPointEmail</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">VERIFICAR NO T01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operacao administrativa padrao</t>
+          <t xml:space="preserve">Se existir, o tipo de uso separa faturacao de comercial sem criar campo</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">N13</t>
+          <t xml:space="preserve">N11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-20 carga massiva</t>
+          <t xml:space="preserve">RN-16, CA-11 chaves de coincidencia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Loader e Bulk API</t>
+          <t xml:space="preserve">Matching Rules</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2127,267 +2364,267 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacidade padrao. A HU so fixa a regra</t>
+          <t xml:space="preserve">Esta HU define as chaves, a HU-006 configura</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">N14</t>
+          <t xml:space="preserve">N12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-23, CA-14 aprovacao de dado sensivel</t>
+          <t xml:space="preserve">RN-18 fusao de duplicados</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDM_Conta_Sensivel e AprobacionDatosSensiblesCuenta</t>
+          <t xml:space="preserve">Merge nativo, inclusive Person Account</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">JA EXISTE E ESTA ATIVO</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mais Aprobador_Config__mdt, SensitiveDataApprover__mdt e o permission set MDG Aprobador. Praticamente entregue</t>
+          <t xml:space="preserve">Operacao administrativa padrao</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">N15</t>
+          <t xml:space="preserve">N13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-24, CA-13 auditoria</t>
+          <t xml:space="preserve">RN-20 carga massiva</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Field History Tracking</t>
+          <t xml:space="preserve">Data Loader e Bulk API</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR PARCIAL</t>
+          <t xml:space="preserve">REUSAR</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teto de 20 campos por objeto. Field Audit Trail nao licenciado</t>
+          <t xml:space="preserve">Capacidade padrao. A HU so fixa a regra</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">N16</t>
+          <t xml:space="preserve">N14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25, CA-15 visibilidade por sociedade</t>
+          <t xml:space="preserve">RN-23, CA-14 aprovacao de dado sensivel</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restriction Rules</t>
+          <t xml:space="preserve">MDM_Conta_Sensivel e AprobacionDatosSensiblesCuenta</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO SERVE</t>
+          <t xml:space="preserve">JA EXISTE E ESTA ATIVO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nao cobre Account. Disponivel so para objetos custom, external, contratos, eventos, tarefas e time sheets</t>
+          <t xml:space="preserve">Mais Aprobador_Config__mdt, SensitiveDataApprover__mdt e o permission set MDG Aprobador. Praticamente entregue</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">N17</t>
+          <t xml:space="preserve">N15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25 visibilidade por sociedade</t>
+          <t xml:space="preserve">RN-24, CA-13 auditoria</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sharing Rule por criterio</t>
+          <t xml:space="preserve">Field History Tracking</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO SERVE</t>
+          <t xml:space="preserve">REUSAR PARCIAL</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">So le campo da propria conta, e a RN-05 proibe campo de sociedade na conta</t>
+          <t xml:space="preserve">Teto de 20 campos por objeto. Field Audit Trail nao licenciado</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">N18</t>
+          <t xml:space="preserve">N16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25, Escenario 7 visibilidade por sociedade</t>
+          <t xml:space="preserve">RN-25, CA-15 visibilidade por sociedade</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apex managed sharing sobre AccountShare</t>
+          <t xml:space="preserve">Restriction Rules</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONSTRUIR</t>
+          <t xml:space="preserve">NAO SERVE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unico caminho que nao contradiz a RN-05. E codigo com teste, muda a estimativa</t>
+          <t xml:space="preserve">Nao cobre Account. Disponivel so para objetos custom, external, contratos, eventos, tarefas e time sheets</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">N19</t>
+          <t xml:space="preserve">N17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-29 protecao de dado sensivel</t>
+          <t xml:space="preserve">RN-25 visibilidade por sociedade</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLS e masking</t>
+          <t xml:space="preserve">Sharing Rule por criterio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">NAO SERVE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cobre visibilidade. Nao cobre cifra at rest, que exige Shield e nao esta licenciado</t>
+          <t xml:space="preserve">So le campo da propria conta, e a RN-05 proibe campo de sociedade na conta</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">N20</t>
+          <t xml:space="preserve">N18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-30 retencao e anonimizacao</t>
+          <t xml:space="preserve">RN-25, Escenario 7 visibilidade por sociedade</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Privacy Center</t>
+          <t xml:space="preserve">Flow que estampa a marca mais criteria-based sharing rule</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">NAO LICENCIADO</t>
+          <t xml:space="preserve">CONSTRUIR DECLARATIVO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Versao nativa da plataforma faz retencao e mascaramento, mas e add on pago</t>
+          <t xml:space="preserve">E o contorno que a propria doc de sharing rule indica para campo nao suportado: automacao mantem um campo texto ou checkbox, a regra le o campo. Zero Apex</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">N21</t>
+          <t xml:space="preserve">N18b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-31, CA-16 documentos</t>
+          <t xml:space="preserve">RN-25 visibilidade por sociedade</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salesforce Files e ContentDocumentLink</t>
+          <t xml:space="preserve">Flow criando AccountShare direto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">DESCARTADO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Falta so um campo que marque o principal</t>
+          <t xml:space="preserve">De fora do Apex so se escreve share com RowCause Manual, e share manual e apagado quando o dono muda. Motivo proprio de compartilhamento exige Apex Sharing Reason</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">N22</t>
+          <t xml:space="preserve">N18c</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-33 consentimento</t>
+          <t xml:space="preserve">RN-25 limite de regras</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Individual, ContactPointTypeConsent, DataUsePurpose</t>
+          <t xml:space="preserve">300 sharing rules por objeto, 50 por criterio</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">CABE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exige a preferencia Data Protection and Privacy habilitada. Tem BusinessBrandId, entao consentimento por marca e nativo</t>
+          <t xml:space="preserve">14 sociedades cabem com folga nas duas variantes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">N23</t>
+          <t xml:space="preserve">N19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-26, RN-27 erro de replicacao</t>
+          <t xml:space="preserve">RN-29 protecao de dado sensivel</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nebula Logger</t>
+          <t xml:space="preserve">FLS e masking</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2397,59 +2634,167 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja instalado. Nao criar campo de log nem contador de retentativa</t>
+          <t xml:space="preserve">Cobre visibilidade. Nao cobre cifra at rest, que exige Shield e nao esta licenciado</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">N24</t>
+          <t xml:space="preserve">N20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-06, CA-05 conta sem dono vendedor</t>
+          <t xml:space="preserve">RN-30 retencao e anonimizacao</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dono padrao e fila</t>
+          <t xml:space="preserve">Privacy Center</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">REUSAR</t>
+          <t xml:space="preserve">NAO LICENCIADO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configuracao, nao construcao</t>
+          <t xml:space="preserve">Versao nativa da plataforma faz retencao e mascaramento, mas e add on pago</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">N21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-31, CA-16 documentos</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Salesforce Files e ContentDocumentLink</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Falta so um campo que marque o principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-33 consentimento</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individual, ContactPointTypeConsent, DataUsePurpose</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exige a preferencia Data Protection and Privacy habilitada. Tem BusinessBrandId, entao consentimento por marca e nativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-26, RN-27 erro de replicacao</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nebula Logger</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ja instalado. Nao criar campo de log nem contador de retentativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-06, CA-05 conta sem dono vendedor</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dono padrao e fila</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REUSAR</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Configuracao, nao construcao</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t xml:space="preserve">N25</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t xml:space="preserve">RN-09 pedido nao altera o maestro</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t xml:space="preserve">Regra de processo</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t xml:space="preserve">NAO CONSTRUIR</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t xml:space="preserve">E criterio de desenho, nao componente</t>
         </is>

</xml_diff>

<commit_message>
HU-017: as consideracoes oficiais de sharing rule e de Repeater, e o acesso implicito pela conta pai
</commit_message>
<xml_diff>
--- a/docs/hu017/HU017_Tarefas_Tecnicas.xlsx
+++ b/docs/hu017/HU017_Tarefas_Tecnicas.xlsx
@@ -444,7 +444,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedir apenas os dados locais faltantes e criar o registro de relacao, sem gerar novo identificador maestro. Usar componentes reativos, GA no Winter 24. Sem LWC. Se precisar de mais de uma sociedade por vez, avaliar o Repeater, lembrando que componente reativo nao funciona dentro dele</t>
+          <t xml:space="preserve">Pedir apenas os dados locais faltantes e criar o registro de relacao, sem gerar novo identificador maestro. Componentes reativos, GA no Winter 24, e sem LWC. A lista de sociedades onde o cliente ainda NAO esta estendido sai de um Collection Choice Set calculado antes da tela, porque Choice Option nao e reativa</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -466,116 +466,116 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">T10</t>
+          <t xml:space="preserve">T09a</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aposentar Account.Sociedad__c</t>
+          <t xml:space="preserve">Subir os flows para API 59.0 ou superior</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Divida</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account.Sociedad__c (TEXTAREA)</t>
+          <t xml:space="preserve">Versao de API dos flows da HU</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo de sociedade em texto livre na conta, que contradiz a RN-05 e nao tem integridade. Fazer backfill para AccountAccountRelation, repontar o que usa e desativar. Nao sincronizar os dois por Flow</t>
+          <t xml:space="preserve">A preferencia de opt in da beta de componentes reativos expira. Sem API 59.0 a reatividade da tela nao vale</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">T08</t>
+          <t xml:space="preserve">T09</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-05, Governanca</t>
+          <t xml:space="preserve">RN-05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACHADO 18/08</t>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">T11</t>
+          <t xml:space="preserve">T10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente sem vendedor proprietario</t>
+          <t xml:space="preserve">Aposentar Account.Sociedad__c</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup</t>
+          <t xml:space="preserve">Divida</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, dono padrao</t>
+          <t xml:space="preserve">Account.Sociedad__c (TEXTAREA)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Definir dono padrao da conta como usuario ou fila de dados maestros, nunca o assessor. O assessor se associa ao documento comercial</t>
+          <t xml:space="preserve">Campo de sociedade em texto livre na conta, que contradiz a RN-05 e nao tem integridade. Fazer backfill para AccountAccountRelation, repontar o que usa e desativar. Nao sincronizar os dois por Flow</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T08</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-06, CA-05</t>
+          <t xml:space="preserve">RN-05, Governanca</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">ACHADO 18/08</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">T12</t>
+          <t xml:space="preserve">T11</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente originador e terceiro faturado</t>
+          <t xml:space="preserve">Cliente sem vendedor proprietario</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account ou Quote, relacao entre as partes</t>
+          <t xml:space="preserve">Account, dono padrao</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrar quem negocia e quem fatura quando forem diferentes, conservando o usuario final do veiculo. Verificar antes se AccountAccountRelation ja serve</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T08</t>
+          <t xml:space="preserve">Definir dono padrao da conta como usuario ou fila de dados maestros, nunca o assessor. O assessor se associa ao documento comercial</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-07</t>
+          <t xml:space="preserve">RN-06, CA-05</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -587,37 +587,37 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">T13</t>
+          <t xml:space="preserve">T12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baixa logica do cliente</t>
+          <t xml:space="preserve">Cliente originador e terceiro faturado</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField mais Flow</t>
+          <t xml:space="preserve">CustomField</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account: estado e vigencia</t>
+          <t xml:space="preserve">Account ou Quote, relacao entre as partes</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inativar por estado ou data, tirar das list views operativas e conservar o historico. Sem exclusao fisica. Checar antes se ha campo de estado em Account</t>
+          <t xml:space="preserve">Registrar quem negocia e quem fatura quando forem diferentes, conservando o usuario final do veiculo. Verificar antes se AccountAccountRelation ja serve</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">T01</t>
+          <t xml:space="preserve">T08</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-10, CA-17, Escenario 9</t>
+          <t xml:space="preserve">RN-07</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -629,61 +629,66 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 2</t>
+          <t xml:space="preserve">T13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">QUALIDADE DO DADO</t>
+          <t xml:space="preserve">Baixa logica do cliente</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CustomField mais Flow</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account: estado e vigencia</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inativar por estado ou data, tirar das list views operativas e conservar o historico. Sem exclusao fisica. Checar antes se ha campo de estado em Account</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T01</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-10, CA-17, Escenario 9</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">BLOCO 2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tabela de regras de documento por pais</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CustomMetadata</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DocumentRuleByCountry</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tipos de documento admitidos e formato por pais, editavel em Setup sem desenvolvimento. Uma linha por pais e tipo</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN-12, RN-21, CA-07</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">QUALIDADE DO DADO</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">T15</t>
+          <t xml:space="preserve">T14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tabela de regras de telefone por pais</t>
+          <t xml:space="preserve">Tabela de regras de documento por pais</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -693,17 +698,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">PhoneRuleByCountry</t>
+          <t xml:space="preserve">DocumentRuleByCountry</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prefixo, comprimento e digito inicial de movel por pais</t>
+          <t xml:space="preserve">Tipos de documento admitidos e formato por pais, editavel em Setup sem desenvolvimento. Uma linha por pais e tipo</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-14, CA-09</t>
+          <t xml:space="preserve">RN-12, RN-21, CA-07</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -715,37 +720,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">T16</t>
+          <t xml:space="preserve">T15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validacao de documento e telefone</t>
+          <t xml:space="preserve">Tabela de regras de telefone por pais</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">ValidationRule ou Flow</t>
+          <t xml:space="preserve">CustomMetadata</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account</t>
+          <t xml:space="preserve">PhoneRuleByCountry</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aplicar as duas tabelas na gravacao e informar o formato esperado quando falhar. Description ate 255 caracteres</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T14, T15</t>
+          <t xml:space="preserve">Prefixo, comprimento e digito inicial de movel por pais</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-12, RN-14, Escenario 3</t>
+          <t xml:space="preserve">RN-14, CA-09</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -757,37 +757,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">T17</t>
+          <t xml:space="preserve">T16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correio de faturacao separado do comercial</t>
+          <t xml:space="preserve">Validacao de documento e telefone</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decision mais CustomField</t>
+          <t xml:space="preserve">ValidationRule ou Flow</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">ContactPointEmail nativo, ou campo em Account</t>
+          <t xml:space="preserve">Account</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decidir com o T01. Se ContactPointEmail existir, usar o tipo de uso para separar faturacao de comercial em vez de criar campo</t>
+          <t xml:space="preserve">Aplicar as duas tabelas na gravacao e informar o formato esperado quando falhar. Description ate 255 caracteres</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">T01</t>
+          <t xml:space="preserve">T14, T15</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-13, CA-08</t>
+          <t xml:space="preserve">RN-12, RN-14, Escenario 3</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -799,37 +799,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">T18</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exigir o correio de faturacao so onde aplica</t>
+          <t xml:space="preserve">Correio de faturacao separado do comercial</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic Forms</t>
+          <t xml:space="preserve">Decision mais CustomField</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pagina de Account</t>
+          <t xml:space="preserve">ContactPointEmail nativo, ou campo em Account</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcar o campo como obrigatorio por regra de visibilidade quando o pais exigir faturacao eletronica, e esconder onde nao aplica. Condicionar campo a campo, nunca a secao, porque regra de secao so e avaliada depois de salvar</t>
+          <t xml:space="preserve">Decidir com o T01. Se ContactPointEmail existir, usar o tipo de uso para separar faturacao de comercial em vez de criar campo</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">T17</t>
+          <t xml:space="preserve">T01</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-13, Escenario 4</t>
+          <t xml:space="preserve">RN-13, CA-08</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -841,12 +841,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">T19</t>
+          <t xml:space="preserve">T18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obrigatoriedade configuravel por pais, sociedade e tipo</t>
+          <t xml:space="preserve">Exigir o correio de faturacao so onde aplica</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -856,22 +856,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pagina de Account por Record Type</t>
+          <t xml:space="preserve">Pagina de Account</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Montar as regras de obrigatoriedade em Dynamic Forms, que desde Winter 23 suporta Person Account. Sem desenvolvimento e sem codigo</t>
+          <t xml:space="preserve">Marcar o campo como obrigatorio por regra de visibilidade quando o pais exigir faturacao eletronica, e esconder onde nao aplica. Condicionar campo a campo, nunca a secao, porque regra de secao so e avaliada depois de salvar</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">T03</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-11, CA-06</t>
+          <t xml:space="preserve">RN-13, Escenario 4</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -883,32 +883,37 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">T20</t>
+          <t xml:space="preserve">T19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Normalizacao antes de gravar</t>
+          <t xml:space="preserve">Obrigatoriedade configuravel por pais, sociedade e tipo</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow</t>
+          <t xml:space="preserve">Dynamic Forms</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, before save</t>
+          <t xml:space="preserve">Pagina de Account por Record Type</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Normalizar nome, documento, telefone, correio e endereco antes de gravar, para as regras de coincidencia operarem sobre valores comparaveis</t>
+          <t xml:space="preserve">Montar as regras de obrigatoriedade em Dynamic Forms, que desde Winter 23 suporta Person Account. Sem desenvolvimento e sem codigo</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T03</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-15, CA-10</t>
+          <t xml:space="preserve">RN-11, CA-06</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -920,37 +925,32 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">T21</t>
+          <t xml:space="preserve">T20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Definir as chaves de coincidencia</t>
+          <t xml:space="preserve">Normalizacao antes de gravar</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentacao</t>
+          <t xml:space="preserve">Flow</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entrega para a HU-006</t>
+          <t xml:space="preserve">Account, before save</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exata sobre documento mais pais, difusa sobre nome, correio, telefone e razao social. Esta HU define, a HU-006 configura</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T04</t>
+          <t xml:space="preserve">Normalizar nome, documento, telefone, correio e endereco antes de gravar, para as regras de coincidencia operarem sobre valores comparaveis</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-16, CA-11</t>
+          <t xml:space="preserve">RN-15, CA-10</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -962,27 +962,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">T22</t>
+          <t xml:space="preserve">T21</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fechar o furo de compartilhamento na Duplicate Rule</t>
+          <t xml:space="preserve">Definir as chaves de coincidencia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup</t>
+          <t xml:space="preserve">Documentacao</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuplicateRule de Account, securityOption</t>
+          <t xml:space="preserve">Entrega para a HU-006</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Com EnforceSharingRules o insert passa em silencio quando o usuario nao enxerga o duplicado. Decidir entre BypassSharingRules, que revela existencia, e depender do campo unico do T04</t>
+          <t xml:space="preserve">Exata sobre documento mais pais, difusa sobre nome, correio, telefone e razao social. Esta HU define, a HU-006 configura</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-17, CA-01, CA-12</t>
+          <t xml:space="preserve">RN-16, CA-11</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1004,32 +1004,37 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">T23</t>
+          <t xml:space="preserve">T22</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registro incompleto nao persiste</t>
+          <t xml:space="preserve">Fechar o furo de compartilhamento na Duplicate Rule</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, depuracao</t>
+          <t xml:space="preserve">DuplicateRule de Account, securityOption</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Depurar os registros cuja criacao nao se completou ou ficaram em erro de integracao</t>
+          <t xml:space="preserve">Com EnforceSharingRules o insert passa em silencio quando o usuario nao enxerga o duplicado. Decidir entre BypassSharingRules, que revela existencia, e depender do campo unico do T04</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T04</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-19, CA-19</t>
+          <t xml:space="preserve">RN-17, CA-01, CA-12</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1041,66 +1046,61 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 3</t>
+          <t xml:space="preserve">T23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">GOVERNANCA DO DADO</t>
+          <t xml:space="preserve">Registro incompleto nao persiste</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flow</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account, depuracao</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Depurar os registros cuja criacao nao se completou ou ficaram em erro de integracao</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-19, CA-19</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">T24</t>
+          <t xml:space="preserve">BLOCO 3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusar as aprovacoes de dado sensivel</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reuso</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MDM_Conta_Sensivel e AprobacionDatosSensiblesCuenta</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partir dos dois processos que ja estao ativos em Account. Ajustar apenas os campos que disparam, conforme a RN-23: nome, documento, endereco fiscal, correio de faturacao e telefone principal</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T02</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN-23, CA-14</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JA EXISTE, ajustar</t>
+          <t xml:space="preserve">GOVERNANCA DO DADO</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">T25</t>
+          <t xml:space="preserve">T24</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reusar Aprobador_Config__mdt</t>
+          <t xml:space="preserve">Reusar as aprovacoes de dado sensivel</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1110,54 +1110,54 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aprobador_Config__mdt e SensitiveDataApprover__mdt</t>
+          <t xml:space="preserve">MDM_Conta_Sensivel e AprobacionDatosSensiblesCuenta</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usar o metadata de aprovador que ja existe para determinar o avaliador por tipo de dado, sociedade e papel</t>
+          <t xml:space="preserve">Partir dos dois processos que ja estao ativos em Account. Ajustar apenas os campos que disparam, conforme a RN-23: nome, documento, endereco fiscal, correio de faturacao e telefone principal</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">T24</t>
+          <t xml:space="preserve">T02</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-23</t>
+          <t xml:space="preserve">RN-23, CA-14</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">JA EXISTE</t>
+          <t xml:space="preserve">JA EXISTE, ajustar</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">T26</t>
+          <t xml:space="preserve">T25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historico de campo nos campos priorizados</t>
+          <t xml:space="preserve">Reusar Aprobador_Config__mdt</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Object Manager</t>
+          <t xml:space="preserve">Reuso</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, Field History Tracking</t>
+          <t xml:space="preserve">Aprobador_Config__mdt e SensitiveDataApprover__mdt</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selecionar ate 20 campos, comecando pelos sensiveis da RN-23. Field Audit Trail nao esta licenciado e a propria HU reconhece</t>
+          <t xml:space="preserve">Usar o metadata de aprovador que ja existe para determinar o avaliador por tipo de dado, sociedade e papel</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1167,44 +1167,49 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-24, CA-13</t>
+          <t xml:space="preserve">RN-23</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">JA EXISTE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27</t>
+          <t xml:space="preserve">T26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">OWD de Account privada</t>
+          <t xml:space="preserve">Historico de campo nos campos priorizados</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup</t>
+          <t xml:space="preserve">Object Manager</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Organization Wide Defaults</t>
+          <t xml:space="preserve">Account, Field History Tracking</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deixar Account como Private. Sharing rule concede acesso e nunca restringe, entao sem OWD privada a RN-25 nao se sustenta</t>
+          <t xml:space="preserve">Selecionar ate 20 campos, comecando pelos sensiveis da RN-23. Field Audit Trail nao esta licenciado e a propria HU reconhece</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T24</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25, CA-15</t>
+          <t xml:space="preserve">RN-24, CA-13</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1216,32 +1221,32 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27a</t>
+          <t xml:space="preserve">T27</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificar o operador do criterio de sharing rule</t>
+          <t xml:space="preserve">OWD de Account privada</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificacao</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Setup, Sharing Settings</t>
+          <t xml:space="preserve">Organization Wide Defaults</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abrir uma criteria-based sharing rule de Account e ver se o operador contains esta disponivel para campo texto. Decide entre um campo texto com 14 regras ou 14 checkbox com 14 regras</t>
+          <t xml:space="preserve">Deixar Account como Private. Sharing rule concede acesso e nunca restringe, entao sem OWD privada a RN-25 nao se sustenta</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25</t>
+          <t xml:space="preserve">RN-25, CA-15</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1253,37 +1258,32 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27b</t>
+          <t xml:space="preserve">T27a</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca das sociedades habilitadas na conta</t>
+          <t xml:space="preserve">Verificar o operador do criterio de sharing rule</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField</t>
+          <t xml:space="preserve">Verificacao</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, um checkbox por sociedade, ou um texto com a lista</t>
+          <t xml:space="preserve">Setup, Sharing Settings</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Criar a marca que a sharing rule vai ler. Nao e a chave maestra, e derivado da AccountAccountRelation, entao nao conflita com a unicidade da RN-05. Confirmar essa leitura com a Melisa antes de empacotar</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T27a</t>
+          <t xml:space="preserve">Abrir uma criteria-based sharing rule de Account e ver se o operador contains esta disponivel para campo texto. Decide entre um campo texto com 14 regras ou 14 checkbox com 14 regras</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-05, RN-25</t>
+          <t xml:space="preserve">RN-25</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1295,32 +1295,32 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27c</t>
+          <t xml:space="preserve">T27b</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow que estampa a marca de sociedade</t>
+          <t xml:space="preserve">Marca das sociedades habilitadas na conta</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow</t>
+          <t xml:space="preserve">CustomField</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">AccountAccountRelation, apos criar, atualizar e excluir</t>
+          <t xml:space="preserve">Account, um checkbox por sociedade, ou um texto com a lista</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manter a marca da T27b sincronizada com os registros de relacao. E o contorno que a propria documentacao de sharing rule indica: automacao mantem o campo, a regra le o campo</t>
+          <t xml:space="preserve">Criar a marca que a sharing rule vai ler. Nao e a chave maestra, e derivado da AccountAccountRelation, entao nao conflita com a unicidade da RN-05. Confirmar essa leitura com a Melisa antes de empacotar</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27b</t>
+          <t xml:space="preserve">T27a</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1337,32 +1337,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27d</t>
+          <t xml:space="preserve">T27c</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Public group por sociedade</t>
+          <t xml:space="preserve">Flow que estampa a marca de sociedade</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Group</t>
+          <t xml:space="preserve">Flow</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Um public group por sociedade</t>
+          <t xml:space="preserve">AccountAccountRelation, apos criar, atualizar e excluir</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Criar o grupo que recebe o acesso em cada regra, e definir quem entra em cada um</t>
+          <t xml:space="preserve">Manter a marca da T27b sincronizada com os registros de relacao. E o contorno que a propria documentacao de sharing rule indica: automacao mantem o campo, a regra le o campo</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27b</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25</t>
+          <t xml:space="preserve">RN-05, RN-25</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1374,37 +1379,32 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27e</t>
+          <t xml:space="preserve">T27d</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Criteria-based sharing rules por sociedade</t>
+          <t xml:space="preserve">Public group por sociedade</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">SharingRules</t>
+          <t xml:space="preserve">Group</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, uma regra por sociedade</t>
+          <t xml:space="preserve">Um public group por sociedade</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uma regra por sociedade lendo a marca da T27b e concedendo ao grupo da T27d. Teto de 50 regras por criterio por objeto, e 14 sociedades cabem</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T27b, T27c, T27d</t>
+          <t xml:space="preserve">Criar os grupos ANTES das regras. O Share With de uma sharing rule nao pode ser editado depois de salvar, so apagando e recriando a regra</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25, Escenario 7</t>
+          <t xml:space="preserve">RN-25</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1416,37 +1416,37 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27f</t>
+          <t xml:space="preserve">T27e</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medir o recalculo de compartilhamento</t>
+          <t xml:space="preserve">Criteria-based sharing rules por sociedade</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verificacao</t>
+          <t xml:space="preserve">SharingRules</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antes da carga inicial</t>
+          <t xml:space="preserve">Account, uma regra por sociedade</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atualizar a marca em volume dispara recalculo assincrono de compartilhamento. Medir com a base real antes da carga de clientes</t>
+          <t xml:space="preserve">Uma regra por sociedade lendo a marca da T27b e concedendo ao grupo da T27d. Teto de 50 regras por criterio por objeto, e 14 sociedades cabem. Decidir ANTES de salvar a opcao Include records owned by users who cannot have an assigned role, que vem marcada e nao pode ser editada depois</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27e</t>
+          <t xml:space="preserve">T27b, T27c, T27d</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-25</t>
+          <t xml:space="preserve">RN-25, Escenario 7</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1458,37 +1458,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">T28</t>
+          <t xml:space="preserve">T27f</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo de permissoes e FLS</t>
+          <t xml:space="preserve">Diferir o recalculo na carga inicial</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PermissionSet mais FLS</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">MasterDataAdmin, MasterDataRead</t>
+          <t xml:space="preserve">Defer Sharing Calculations</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Separar quem administra o maestro de quem so cria e atualiza dentro do perfil, com FLS nos campos sensiveis</t>
+          <t xml:space="preserve">Ligar o Defer Sharing Calculations antes da carga em massa de clientes e recalcular depois. E o remedio que a propria documentacao recomenda para atualizacao em larga escala</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">T27</t>
+          <t xml:space="preserve">T27e</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-22, RN-25, CA-15</t>
+          <t xml:space="preserve">RN-25</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1500,74 +1500,79 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">T29</t>
+          <t xml:space="preserve">T27g</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marca de nao sincronizado com SAP</t>
+          <t xml:space="preserve">Declarar o acesso implicito pela conta pai</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField</t>
+          <t xml:space="preserve">Documentacao</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account: estado de sincronizacao e ultimo erro</t>
+          <t xml:space="preserve">Risco a escrever na HU</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcar o cliente como nao sincronizado quando a replicacao falhar. Registrar o erro no Nebula Logger pela acao invocavel de Flow, sem escrever Apex e sem criar campo de log</t>
+          <t xml:space="preserve">Quem tem acesso a uma Opportunity, Case ou Contact ganha visibilidade da conta pai. Entao o Escenario 7 nao e hermetico: o assessor ve o cliente pelo negocio que e dele, independente da sociedade. Escrever na HU antes de UAT. Se o negocio quiser hermetismo, a restricao sobe para Opportunity, Quote e Order, e isso e outra historia</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T27e</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-26, RN-27, CA-18, Escenario 8</t>
+          <t xml:space="preserve">RN-25, Escenario 7</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">A DECLARAR</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T30</t>
+          <t xml:space="preserve">T28</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atributos fiscais derivados por regra</t>
+          <t xml:space="preserve">Modelo de permissoes e FLS</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow ou ExpressionSet</t>
+          <t xml:space="preserve">PermissionSet mais FLS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, derivacao automatica</t>
+          <t xml:space="preserve">MasterDataAdmin, MasterDataRead</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivar tipo de imposto, condicao de pagamento, classificacao B2C ou B2B, grupo de contas e lista de precos a partir do tipo de documento e de cliente. Nao se mostram na captura e sao sensiveis para a replicacao</t>
+          <t xml:space="preserve">Separar quem administra o maestro de quem so cria e atualiza dentro do perfil, com FLS nos campos sensiveis</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">T27</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-32</t>
+          <t xml:space="preserve">RN-22, RN-25, CA-15</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -1579,44 +1584,74 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 4</t>
+          <t xml:space="preserve">T29</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROTECAO DO DADO</t>
+          <t xml:space="preserve">Marca de nao sincronizado com SAP</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CustomField</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account: estado de sincronizacao e ultimo erro</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcar o cliente como nao sincronizado quando a replicacao falhar. Registrar o erro no Nebula Logger pela acao invocavel de Flow, sem escrever Apex e sem criar campo de log</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-26, RN-27, CA-18, Escenario 8</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">T31</t>
+          <t xml:space="preserve">T30</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento de respaldo com principal</t>
+          <t xml:space="preserve">Atributos fiscais derivados por regra</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">CustomField mais Files</t>
+          <t xml:space="preserve">Flow ou ExpressionSet</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account, marcacao de documento principal</t>
+          <t xml:space="preserve">Account, derivacao automatica</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guardar identificacao, registro tributario e poderes como Files, com um campo que marque o principal. O expediente comercial e da HU-078</t>
+          <t xml:space="preserve">Derivar tipo de imposto, condicao de pagamento, classificacao B2C ou B2B, grupo de contas e lista de precos a partir do tipo de documento e de cliente. Nao se mostram na captura e sao sensiveis para a replicacao</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T14</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-31, CA-16</t>
+          <t xml:space="preserve">RN-32</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -1628,79 +1663,44 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">BLOCO 4</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ligar Data Protection and Privacy</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Setup</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Objetos de consentimento</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Os objetos de consentimento so existem com a preferencia habilitada. Ligar antes de a HU-034 precisar</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T01</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RN-33</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">PROTECAO DO DADO</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">T33</t>
+          <t xml:space="preserve">T31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consentimento como dado do cliente</t>
+          <t xml:space="preserve">Documento de respaldo com principal</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reuso</t>
+          <t xml:space="preserve">CustomField mais Files</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Individual, ContactPointTypeConsent</t>
+          <t xml:space="preserve">Account, marcacao de documento principal</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guardar consentimento e canal de preferencia nos objetos nativos. ContactPointTypeConsent tem BusinessBrandId, entao consentimento por marca sai nativo, o que importa num grupo multimarca</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T32</t>
+          <t xml:space="preserve">Guardar identificacao, registro tributario e poderes como Files, com um campo que marque o principal. O expediente comercial e da HU-078</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-33</t>
+          <t xml:space="preserve">RN-31, CA-16</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -1712,74 +1712,79 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">T34</t>
+          <t xml:space="preserve">T32</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Declarar o que depende de licenca nao contratada</t>
+          <t xml:space="preserve">Ligar Data Protection and Privacy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentacao</t>
+          <t xml:space="preserve">Setup</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Riscos da HU</t>
+          <t xml:space="preserve">Objetos de consentimento</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cifrado at rest exige Shield e retencao com anonimizacao exige Privacy Center, nenhum dos dois licenciado. FLS e masking cobrem visibilidade e nao substituem cifra. Registrar como premissa, nao como tarefa</t>
+          <t xml:space="preserve">Os objetos de consentimento so existem com a preferencia habilitada. Ligar antes de a HU-034 precisar</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T01</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-29, RN-30</t>
+          <t xml:space="preserve">RN-33</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOQUEADO</t>
+          <t xml:space="preserve">A FAZER</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">T35</t>
+          <t xml:space="preserve">T33</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nao usar Dynamic Forms como seguranca</t>
+          <t xml:space="preserve">Consentimento como dado do cliente</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Padrao</t>
+          <t xml:space="preserve">Reuso</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisao das paginas</t>
+          <t xml:space="preserve">Individual, ContactPointTypeConsent</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Campo escondido por regra de visibilidade continua acessivel em relatorio, list view e API. Proteger dado sensivel so por FLS</t>
+          <t xml:space="preserve">Guardar consentimento e canal de preferencia nos objetos nativos. ContactPointTypeConsent tem BusinessBrandId, entao consentimento por marca sai nativo, o que importa num grupo multimarca</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">T19</t>
+          <t xml:space="preserve">T32</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t xml:space="preserve">RN-29</t>
+          <t xml:space="preserve">RN-33</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -1791,24 +1796,49 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLOCO 5</t>
+          <t xml:space="preserve">T34</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">MULTI PAIS E FECHAMENTO</t>
+          <t xml:space="preserve">Declarar o que depende de licenca nao contratada</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentacao</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Riscos da HU</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cifrado at rest exige Shield e retencao com anonimizacao exige Privacy Center, nenhum dos dois licenciado. FLS e masking cobrem visibilidade e nao substituem cifra. Registrar como premissa, nao como tarefa</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RN-29, RN-30</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLOQUEADO</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">T36</t>
+          <t xml:space="preserve">T35</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pais e dimensao de dado, nunca nome de metadado</t>
+          <t xml:space="preserve">Nao usar Dynamic Forms como seguranca</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1818,22 +1848,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revisao de nomenclatura</t>
+          <t xml:space="preserve">Revisao das paginas</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">As regras por pais vivem nas tabelas do T14 e T15. Nenhum campo, flow ou classe com pais no API name</t>
+          <t xml:space="preserve">Campo escondido por regra de visibilidade continua acessivel em relatorio, list view e API. Proteger dado sensivel so por FLS</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">T14</t>
+          <t xml:space="preserve">T19</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Convencao GRPQM</t>
+          <t xml:space="preserve">RN-29</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -1845,79 +1875,49 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">T37</t>
+          <t xml:space="preserve">BLOCO 5</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Translation</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Translation Workbench</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Traduzir campos, valores de picklist, Record Types e mensagens de erro criados nesta HU</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">T16</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Convencao GRPQM</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A FAZER</t>
+          <t xml:space="preserve">MULTI PAIS E FECHAMENTO</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">T38</t>
+          <t xml:space="preserve">T36</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order nos flows criados</t>
+          <t xml:space="preserve">Pais e dimensao de dado, nunca nome de metadado</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Object Manager</t>
+          <t xml:space="preserve">Padrao</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trigger Order de cada flow em Account</t>
+          <t xml:space="preserve">Revisao de nomenclatura</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account ja e um dos objetos com mais automacao na org. Definir a ordem em cada flow novo</t>
+          <t xml:space="preserve">As regras por pais vivem nas tabelas do T14 e T15. Nenhum campo, flow ou classe com pais no API name</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">T20</t>
+          <t xml:space="preserve">T14</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Governanca</t>
+          <t xml:space="preserve">Convencao GRPQM</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -1929,40 +1929,124 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t xml:space="preserve">T37</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir os rotulos para espanhol</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Translation Workbench</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traduzir campos, valores de picklist, Record Types e mensagens de erro criados nesta HU</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T16</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Convencao GRPQM</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T38</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trigger Order nos flows criados</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Object Manager</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trigger Order de cada flow em Account</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Account ja e um dos objetos com mais automacao na org. Definir a ordem em cada flow novo</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T20</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Governanca</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A FAZER</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t xml:space="preserve">T39</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t xml:space="preserve">Testes dos nove escenarios</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t xml:space="preserve">Flow Test</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t xml:space="preserve">Testes dos flows acionados por registro</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t xml:space="preserve">Cobrir os escenarios 1 a 9 com Flow Test, que versiona junto com o flow. Enfase no 1, no 2 e no 7, e o 7 testado com usuario de outra sociedade, nunca com administrador</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t xml:space="preserve">T27e</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t xml:space="preserve">A FAZER</t>
         </is>

</xml_diff>